<commit_message>
consolidate reports into events
Signed-off-by: Tathagata Chakraborti <tchakra2@outlook.com>
</commit_message>
<xml_diff>
--- a/data/forgotten.xlsx
+++ b/data/forgotten.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tchakra2/cnc-fun/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9273712-372E-AF46-86AB-CF22C268727D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B0E8B25-38DF-AF48-B9ED-4147D3C12E1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="34560" windowHeight="21600" activeTab="1" xr2:uid="{91B247F1-4191-D447-A616-0E249F0596B9}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="34560" windowHeight="21600" xr2:uid="{91B247F1-4191-D447-A616-0E249F0596B9}"/>
   </bookViews>
   <sheets>
     <sheet name="forgotten" sheetId="1" r:id="rId1"/>
@@ -8577,6 +8577,9 @@
       <c r="E79" s="5">
         <v>9</v>
       </c>
+      <c r="F79" s="5">
+        <v>3</v>
+      </c>
       <c r="G79" s="5">
         <v>34</v>
       </c>
@@ -43702,7 +43705,9 @@
       <c r="C839" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="E839" s="11"/>
+      <c r="E839" s="11">
+        <v>0</v>
+      </c>
       <c r="F839" s="5">
         <v>2</v>
       </c>
@@ -43723,7 +43728,9 @@
       <c r="C840" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="E840" s="11"/>
+      <c r="E840" s="11">
+        <v>0</v>
+      </c>
       <c r="F840" s="5">
         <v>2</v>
       </c>

</xml_diff>